<commit_message>
Validate complete form grids and publish distinct corrected downloads
</commit_message>
<xml_diff>
--- a/src/tablescan_local/default_templates/staircase_portrait.xlsx
+++ b/src/tablescan_local/default_templates/staircase_portrait.xlsx
@@ -1330,26 +1330,26 @@
       <c r="Q36" s="16"/>
     </row>
     <row r="37" ht="22.200000762939453" customHeight="1">
-      <c r="A37" t="n">
+      <c r="A37" s="15" t="n">
         <f>ROW()-7</f>
         <v>30</v>
       </c>
-      <c r="B37"/>
-      <c r="C37"/>
-      <c r="D37"/>
-      <c r="E37"/>
-      <c r="F37"/>
-      <c r="G37"/>
-      <c r="H37"/>
-      <c r="I37"/>
-      <c r="J37"/>
-      <c r="K37"/>
-      <c r="L37"/>
-      <c r="M37"/>
-      <c r="N37"/>
-      <c r="O37"/>
-      <c r="P37"/>
-      <c r="Q37"/>
+      <c r="B37" s="16"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16"/>
+      <c r="H37" s="16"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
+      <c r="K37" s="16"/>
+      <c r="L37" s="16"/>
+      <c r="M37" s="16"/>
+      <c r="N37" s="16"/>
+      <c r="O37" s="16"/>
+      <c r="P37" s="16"/>
+      <c r="Q37" s="16"/>
     </row>
   </sheetData>
   <mergeCells>

</xml_diff>